<commit_message>
etapa 2 part 1
</commit_message>
<xml_diff>
--- a/merged_data.xlsx
+++ b/merged_data.xlsx
@@ -31,124 +31,118 @@
     <x:t>Sort by</x:t>
   </x:si>
   <x:si>
-    <x:t>Nina Hall</x:t>
+    <x:t>Diana Stone</x:t>
+  </x:si>
+  <x:si>
+    <x:t>davidpatranjel24@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Beyoncé</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vinyl</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Product name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Matt Young</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Country</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Best reviewed</x:t>
+  </x:si>
+  <x:si>
+    <x:t>George Hill</x:t>
   </x:si>
   <x:si>
     <x:t>davidpatranjel@yahoo.com</x:t>
   </x:si>
   <x:si>
-    <x:t>The Beatles</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Vinyl</x:t>
+    <x:t>Classical</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Kyle Moore</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jazz</x:t>
   </x:si>
   <x:si>
     <x:t>Highest discount</x:t>
   </x:si>
   <x:si>
+    <x:t>Laura James</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Thriller</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Most recent</x:t>
+  </x:si>
+  <x:si>
     <x:t>Fiona Clark</x:t>
   </x:si>
   <x:si>
+    <x:t>Pink Floyd</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hannah Scott</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lowest price</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Eminem</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Most favourite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Charlie Kim</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jenna Fox</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Taylor Swift</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Highest price</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Adele</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Brian Lee</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ian Wright</x:t>
+  </x:si>
+  <x:si>
     <x:t>Pop</x:t>
   </x:si>
   <x:si>
-    <x:t>Highest price</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Diana Stone</x:t>
-  </x:si>
-  <x:si>
-    <x:t>davidpatranjel24@gmail.com</x:t>
+    <x:t>Alice Morgan</x:t>
   </x:si>
   <x:si>
     <x:t>Blues</x:t>
   </x:si>
   <x:si>
-    <x:t>CD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Most recent</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Laura James</x:t>
+    <x:t>Reggae</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Oscar Reed</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rock</x:t>
   </x:si>
   <x:si>
     <x:t>Metallica</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Alice Morgan</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Jazz</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lowest price</x:t>
-  </x:si>
-  <x:si>
-    <x:t>George Hill</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Reggae</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hannah Scott</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Country</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Kyle Moore</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Eminem</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Most favourite</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Charlie Kim</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Pink Floyd</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Beyoncé</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Product name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Matt Young</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Best reviewed</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Classical</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Thriller</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Jenna Fox</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Taylor Swift</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Adele</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Brian Lee</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ian Wright</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Oscar Reed</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Rock</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -547,44 +541,44 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
         <x:v>13</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
+      <x:c r="D5" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
         <x:v>19</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
@@ -592,13 +586,13 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
         <x:v>22</x:v>
@@ -618,7 +612,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:5">
@@ -626,305 +620,305 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
         <x:v>26</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:5">
       <x:c r="A9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
+      <x:c r="D9" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="D9" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="E9" s="0" t="s">
-        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:5">
       <x:c r="A10" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:5">
       <x:c r="A11" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:5">
       <x:c r="A12" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:5">
       <x:c r="A13" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:5">
       <x:c r="A14" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:5">
       <x:c r="A15" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:5">
       <x:c r="A16" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:5">
       <x:c r="A17" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:5">
       <x:c r="A18" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:5">
       <x:c r="A19" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:5">
       <x:c r="A20" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:5">
       <x:c r="A21" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:5">
       <x:c r="A22" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C22" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:5">
       <x:c r="A23" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E23" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:5">
       <x:c r="A24" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:5">
       <x:c r="A25" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:5">
@@ -932,203 +926,203 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E26" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:5">
       <x:c r="A27" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C27" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E27" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:5">
       <x:c r="A28" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C28" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E28" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:5">
       <x:c r="A29" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C29" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E29" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:5">
       <x:c r="A30" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C30" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E30" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:5">
       <x:c r="A31" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C31" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E31" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:5">
       <x:c r="A32" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C32" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E32" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:5">
       <x:c r="A33" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C33" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E33" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:5">
       <x:c r="A34" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C34" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E34" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:5">
       <x:c r="A35" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C35" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E35" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:5">
       <x:c r="A36" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C36" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E36" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:5">
       <x:c r="A37" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C37" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E37" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:5">
@@ -1136,50 +1130,50 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C38" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E38" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:5">
       <x:c r="A39" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C39" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E39" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:5">
       <x:c r="A40" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C40" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D40" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E40" s="0" t="s">
         <x:v>26</x:v>
-      </x:c>
-      <x:c r="D40" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E40" s="0" t="s">
-        <x:v>22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>